<commit_message>
paper run 2026-10-13 19:22
</commit_message>
<xml_diff>
--- a/reports/2026-10-13.xlsx
+++ b/reports/2026-10-13.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,92 @@
       </c>
       <c r="K2" t="n">
         <v>26.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-13T13:42:15.353255+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.781</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.00121</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-13T16:08:54.612014+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00109</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26.6</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>26.6</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3147.809999999999</v>
+        <v>3178.809999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,240 +767,275 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>-39.93</v>
+        <v>66.19</v>
       </c>
       <c r="E15" t="n">
-        <v>26.6</v>
+        <v>48.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>213.37</v>
+      </c>
+      <c r="E16" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-39.93</v>
-      </c>
-      <c r="E17" t="n">
-        <v>26.6</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>101.02</v>
+      </c>
+      <c r="E18" t="n">
+        <v>26.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>-39.93</v>
+        <v>85.41</v>
       </c>
       <c r="E19" t="n">
-        <v>26.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>93.13</v>
+      </c>
+      <c r="E20" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>-118.38</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>78.45</v>
+        <v>110.42</v>
       </c>
       <c r="E22" t="n">
-        <v>26.6</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>123.66</v>
+      </c>
+      <c r="E23" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>45.48</v>
+      </c>
+      <c r="E24" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-50.51</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>26.6</v>
+        <v>330.07</v>
+      </c>
+      <c r="E27" t="n">
+        <v>57.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>26.6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>26.6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>26.6</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -936,93 +1057,281 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>26.6</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>48.6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
         <v>26.6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
+        <v>48.6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>26.6</v>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>35.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>